<commit_message>
feat(data): finalize HR roster + cross-artifact 18.3% consistency tests (D3-M7)
</commit_message>
<xml_diff>
--- a/data/acme_robotics/hr_roster_acme.xlsx
+++ b/data/acme_robotics/hr_roster_acme.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes (DRAFT)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -602,7 +602,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>STATUS: DRAFT - authored Day 2 (D2-M6); finalized Day 3 (D3-M7).</t>
+          <t>STATUS: finalized Day 3 (D3-M7); authored Day 2 (D2-M6).</t>
         </is>
       </c>
     </row>

</xml_diff>